<commit_message>
Shortens industry sector capital expenditure financing repayment period
</commit_message>
<xml_diff>
--- a/InputData/indst/RPfFISCC/RPfFISCC Repayment Period for Financed Indst Sector Capital Costs.xlsx
+++ b/InputData/indst/RPfFISCC/RPfFISCC Repayment Period for Financed Indst Sector Capital Costs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\indst\RPfFISCC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\RPfFISCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4DD7B5B-FACB-44B1-82ED-5197E75644B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F5DE737-0AAC-4D3D-9429-0D3D68AB6FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31680" yWindow="2430" windowWidth="24720" windowHeight="13710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -43,15 +43,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>RPfFESCC Repayment Period for Financed Electricity Sector Capital Costs</t>
-  </si>
-  <si>
-    <t>This variable is used with Vensim's DEPRECIATE STRAIGHTLINE function to spread repayment of electricity sector</t>
-  </si>
-  <si>
-    <t>capital costs over a set number of years.</t>
-  </si>
-  <si>
     <t>Unit: years</t>
   </si>
   <si>
@@ -82,7 +73,16 @@
     <t>other processes</t>
   </si>
   <si>
-    <t>GET SOURCE</t>
+    <t>No source</t>
+  </si>
+  <si>
+    <t>This variable defines the number of years over which industrial sector capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">expenditures are repayed to loaners. </t>
+  </si>
+  <si>
+    <t>RPfFESCC Repayment Period for Financed Industry Sector Capital Costs</t>
   </si>
 </sst>
 </file>
@@ -469,114 +469,114 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="93" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4" s="7"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B27" s="2"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
     </row>
@@ -592,82 +592,82 @@
     <tabColor theme="8" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.54296875" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B3" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B4" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B5" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B6" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B7" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B8" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
       <c r="B9" s="3">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjusts industry capital expenditure financing assumptions, uses cost of debt for interest rate rather than cost of capital, adjusts nonenergy expenditures passthrough effects smoothing time
</commit_message>
<xml_diff>
--- a/InputData/indst/RPfFISCC/RPfFISCC Repayment Period for Financed Indst Sector Capital Costs.xlsx
+++ b/InputData/indst/RPfFISCC/RPfFISCC Repayment Period for Financed Indst Sector Capital Costs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\RPfFISCC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\indst\RPfFISCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48C3A4E-991F-4316-9717-64C2D57C68F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0498CA-1CF1-4C4C-8701-CCC7A1340EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="315" yWindow="1380" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2715" yWindow="840" windowWidth="25245" windowHeight="16245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -617,7 +617,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -625,7 +625,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -633,7 +633,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -641,7 +641,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -649,7 +649,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -657,7 +657,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -665,7 +665,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -673,7 +673,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -681,7 +681,7 @@
         <v>16</v>
       </c>
       <c r="B10" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -689,7 +689,7 @@
         <v>17</v>
       </c>
       <c r="B11" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
pushes draft EPS code + input files that correspond to two major updates: 1) aggregates boiler + nonboiler heat demand in industry, then breaks out five explicit temperature bands 2) endogenizes deployment of waste heat recovery and process efficiency using data from Kermeli + others
</commit_message>
<xml_diff>
--- a/InputData/indst/RPfFISCC/RPfFISCC Repayment Period for Financed Indst Sector Capital Costs.xlsx
+++ b/InputData/indst/RPfFISCC/RPfFISCC Repayment Period for Financed Indst Sector Capital Costs.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\indst\RPfFISCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0498CA-1CF1-4C4C-8701-CCC7A1340EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A09518-9D38-4FE3-93C4-0CDFA8163219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2715" yWindow="840" windowWidth="25245" windowHeight="16245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-6930" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="RPfFESCC" sheetId="17" r:id="rId2"/>
+    <sheet name="RPfFISCC" sheetId="17" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Source:</t>
   </si>
@@ -49,18 +49,6 @@
     <t>Time Period</t>
   </si>
   <si>
-    <t>boilers</t>
-  </si>
-  <si>
-    <t>nonboiler low temp</t>
-  </si>
-  <si>
-    <t>nonboiler med temp</t>
-  </si>
-  <si>
-    <t>nonboiler high temp</t>
-  </si>
-  <si>
     <t>cooling</t>
   </si>
   <si>
@@ -89,6 +77,21 @@
   </si>
   <si>
     <t>other nonprocess</t>
+  </si>
+  <si>
+    <t>heat 100 - 200 C</t>
+  </si>
+  <si>
+    <t>heat 200 - 500 C</t>
+  </si>
+  <si>
+    <t>heat &lt; 100 C</t>
+  </si>
+  <si>
+    <t>heat 500 - 1000 C</t>
+  </si>
+  <si>
+    <t>heat &gt; 1000 C</t>
   </si>
 </sst>
 </file>
@@ -475,114 +478,114 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="93" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B4" s="7"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B6" s="8"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B23" s="2"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B27" s="2"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
     </row>
@@ -597,14 +600,14 @@
   <sheetPr>
     <tabColor theme="8" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="1" max="1" width="25.54296875" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -612,88 +615,96 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B7" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B8" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
       <c r="B9" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B10" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B11" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>